<commit_message>
restate EYDAP exit at ATSE close 13.96 per CHANGELOG
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CrgaPArZPtNB2L5JQrusJ2
</commit_message>
<xml_diff>
--- a/reports/tracker.xlsx
+++ b/reports/tracker.xlsx
@@ -1956,7 +1956,7 @@
         </is>
       </c>
       <c r="B32" s="3" t="n">
-        <v>101303.98</v>
+        <v>101316.71</v>
       </c>
       <c r="C32" s="3" t="n">
         <v>0</v>
@@ -1965,10 +1965,10 @@
         <v>10.13</v>
       </c>
       <c r="E32" s="3" t="n">
-        <v>8871.57</v>
+        <v>8884.299999999999</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>101303.98</v>
+        <v>101316.71</v>
       </c>
       <c r="G32" s="2" t="n">
         <v>0</v>
@@ -1981,19 +1981,19 @@
       </c>
       <c r="J32" s="2" t="n"/>
       <c r="K32" s="4" t="n">
-        <v>0.002217</v>
+        <v>0.002343</v>
       </c>
       <c r="L32" s="4" t="n">
-        <v>0.01304</v>
+        <v>0.013167</v>
       </c>
       <c r="M32" s="4" t="n">
         <v>0</v>
       </c>
       <c r="N32" s="4" t="n">
-        <v>0.011781</v>
+        <v>0.011908</v>
       </c>
       <c r="O32" s="4" t="n">
-        <v>0.008517</v>
+        <v>0.008644000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -2477,7 +2477,7 @@
         <v>1</v>
       </c>
       <c r="G3" s="5" t="n">
-        <v>13.94</v>
+        <v>13.96</v>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
@@ -2499,7 +2499,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>PRICE 13.94 = Boerse Stuttgart quote 21 Oct 2026 as proxy for the ATSE close; replace with the ATSE 21 Oct close once the backfill lands and keep the date</t>
+          <t>ATSE close 21 Oct 2026 per Yahoo (backfill); memo W43 used the Stuttgart quote 13.94 as proxy on decision day</t>
         </is>
       </c>
     </row>
@@ -2709,7 +2709,7 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>Exited 2026-10-21 at EUR13.94 (proxy for ATSE close); about +16% in EUR; memos/2026-W43.md</t>
+          <t>Exited 2026-10-21 at EUR13.96 (ATSE close); about +16% in EUR; memos/2026-W43.md</t>
         </is>
       </c>
     </row>
@@ -3105,7 +3105,7 @@
         <v>7992.01</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>8871.57</v>
+        <v>8884.299999999999</v>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
W43-b: lens 3 screen, thesis maintenance, no trades
Supplement to memos/2026-W43.md. Feed audit clean after backfill. Sanepar
(Moro elected, no privatisation commitment) and Light (RJ closed 9 Sep,
R$1.5bn raise done, 3T26 leverage test pending) updated in pipeline.csv.
Lens 3: BASC scheme-arb logged as watchlist with an entry trigger (spread
consumed by the cost model); Kyocera, AJOT and five others rejected with
reasons. BASC.L added to the feed; CHANGELOG records the manual 21 Oct close.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MKnPwR4dHbEao88b6yahuw
</commit_message>
<xml_diff>
--- a/reports/tracker.xlsx
+++ b/reports/tracker.xlsx
@@ -2007,7 +2007,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S4"/>
+  <dimension ref="A1:S5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2304,6 +2304,73 @@
       <c r="Q4" s="2" t="n"/>
       <c r="R4" s="2" t="n"/>
       <c r="S4" s="2" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>BASC:LSE</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Brown Advisory US Smaller Companies (investment trust)</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>equity</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>watchlist</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Fast</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="3" t="n"/>
+      <c r="I5" s="5" t="n">
+        <v>1640</v>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="n"/>
+      <c r="L5" s="3" t="n"/>
+      <c r="M5" s="4" t="n"/>
+      <c r="N5" s="4" t="n"/>
+      <c r="O5" s="5" t="n">
+        <v>1689</v>
+      </c>
+      <c r="P5" s="4" t="n">
+        <v>0.0299</v>
+      </c>
+      <c r="Q5" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="R5" s="2" t="n">
+        <v>71</v>
+      </c>
+      <c r="S5" s="2" t="inlineStr">
+        <is>
+          <t>Entry trigger, not kill: discount &gt;= 5% to last published NAV with scheme on track. If entered: scheme voted down or withdrawn; circular not out by 2026-11-30; discount &lt; 1%</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2556,7 +2623,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2763,7 +2830,11 @@
           <t>2026-W37.md</t>
         </is>
       </c>
-      <c r="N3" s="2" t="n"/>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>Moro (PL) elected governor 4 Oct 2026, first round, no privatisation commitment; XP neutral 16 Sep; still no dated catalyst; memos/2026-W43-b.md</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -2803,7 +2874,7 @@
       <c r="K4" s="2" t="n"/>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>gated</t>
+          <t>gated (3T26 leverage test)</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
@@ -2811,7 +2882,77 @@
           <t>2026-W37.md</t>
         </is>
       </c>
-      <c r="N4" s="2" t="n"/>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>RJ closed 9 Sep 2026; R$1.5bn capital increase done Jul 2026; 2T26 ND/EBITDA 2.85x reported (2.07x ex convertible); emergence test awaits 3T26 balance sheet; memos/2026-W43-b.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Brown Advisory US Smaller Companies</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>BASC:LSE</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>1640</v>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>GBp</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="n">
+        <v>1689</v>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Uncapped cash exit at 99.25% of residual NAV under scheme of reconstruction into JUSC; Saba 16% irrevocable</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Entry trigger: discount &gt;= 5% to last published NAV with scheme on track (net spread then &gt;= 2.5% after the fund cost model). If entered: scheme voted down or withdrawn; circular not out by 2026-11-30; discount &lt; 1%</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>n/a (fast sleeve)</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>watchlist</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>2026-W43-b.md</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>Not entered: at 1640p vs 1702.25p NAV (15 Oct) the gross spread to the 99.25% cash exit is about 2.6% and the fund cost model on a hedged pair takes about 1.5%; fair spread, not a mispricing</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2824,7 +2965,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3010,6 +3151,212 @@
       <c r="F6" s="2" t="inlineStr">
         <is>
           <t>A dated regulatory decision</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Kyocera</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>6971:TSE</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Mechanism exists (JPY500bn KDDI sales FY26-27, JPY200bn buyback FY26, up to JPY500bn more through FY28, Oasis campaign) but no mispricing shown: KDDI stake about JPY1.56tn (13.36% x JPY11.65tn, 18 Sep) against market cap JPY4.69tn leaves the core at about 31x FY26 forecast operating profit of JPY100bn; P/B 1.39</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Core implied value falls below 15x operating profit, or a tender/buyback at a stated discount</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>AVI Japan Opportunity Trust</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>AJOT:LSE</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Uncapped 100% tender at NAV less 2% (RNS 19 Oct 2026) but the record date was 6pm 20 Oct, before this memo; shares bought now cannot tender and the tender itself bounds the discount</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Next annual tender, if the trust survives the GBP100m floor</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Partners Group Private Equity</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>PGPE:LSE</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Wind-down approved 7 Oct 2026 (about three quarters of holders chose cash) but listed private equity is the salary-correlated exposure the mandate excludes; also no distribution timetable</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>User lifts the factor exclusion by dated amendment</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Edinburgh Worldwide</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>EWI:LSE</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Saba-controlled board promises a tender after the SpaceX IPO (12 Jun 2026) and lock-up expiry (about six months), but the discount was about 1% in June 2026: the closer is priced. Tender terms and date not announced</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Discount wider than 5% with the tender terms published</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Liberty Broadband</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>LBRDK:NASDAQ</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Holdco collapse into Charter completed in August 2026, ten months ahead of the 30 Jun 2027 target. Event over</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Vivendi</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>VIV:EPA</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Paris Court of Appeal ruled 8 Jul 2026 that Bollore does not control Vivendi, so no mandatory offer; holdco discount has no closer; stock fell about 10% that day</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>A distribution of the UMG stake or a buyback at NAV is announced with a date</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Lindsell Train IT</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>LTI:LSE</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>20% tender at NAV less 5% completed 16 Oct 2026; event over; residual discount has no closer</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Next tender announced</t>
         </is>
       </c>
     </row>
@@ -3139,7 +3486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F249"/>
+  <dimension ref="A1:F250"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -9878,6 +10225,36 @@
         </is>
       </c>
     </row>
+    <row r="250">
+      <c r="A250" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B250" s="2" t="inlineStr">
+        <is>
+          <t>BASC.L</t>
+        </is>
+      </c>
+      <c r="C250" s="5" t="n">
+        <v>1640</v>
+      </c>
+      <c r="D250" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="E250" s="2" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="F250" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Memo 2026-W44: rights issues, recapitalisations and index events
Lens 4. Paper fast-sleeve buy: 254 LNZ:VIE at EUR 10.70 (28 Oct Vienna close, manual row; Yahoo unreachable from the routine sandbox). Pennon gated on leverage; Eramet and Yellow Cake to watchlist; Genting, Raizen, Unipol rejected; Corteva logged as a lens-0 pointer. Thesis maintenance on EYDAP, Sanepar, Light; ONCO3 OPA injunction logged.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MvZbV2ah23PJENMDPp5Mb9
</commit_message>
<xml_diff>
--- a/reports/tracker.xlsx
+++ b/reports/tracker.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O36"/>
+  <dimension ref="A1:O37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2184,6 +2184,53 @@
         <v>0.008663000000000001</v>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>98345.49000000001</v>
+      </c>
+      <c r="C37" s="3" t="n">
+        <v>3036.82</v>
+      </c>
+      <c r="D37" s="3" t="n">
+        <v>11.11</v>
+      </c>
+      <c r="E37" s="3" t="n">
+        <v>-3048.97</v>
+      </c>
+      <c r="F37" s="3" t="n">
+        <v>101382.31</v>
+      </c>
+      <c r="G37" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H37" s="4" t="n">
+        <v>-0.003024</v>
+      </c>
+      <c r="I37" s="4" t="n">
+        <v>0.005279</v>
+      </c>
+      <c r="J37" s="2" t="n"/>
+      <c r="K37" s="4" t="n">
+        <v>-1e-05</v>
+      </c>
+      <c r="L37" s="4" t="n">
+        <v>0.013823</v>
+      </c>
+      <c r="M37" s="4" t="n">
+        <v>-1e-05</v>
+      </c>
+      <c r="N37" s="4" t="n">
+        <v>0.016847</v>
+      </c>
+      <c r="O37" s="4" t="n">
+        <v>0.008544</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2195,7 +2242,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S4"/>
+  <dimension ref="A1:S8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2375,7 +2422,7 @@
         </is>
       </c>
       <c r="R2" s="2" t="n">
-        <v>-27</v>
+        <v>-28</v>
       </c>
       <c r="S2" s="2" t="inlineStr">
         <is>
@@ -2492,6 +2539,248 @@
       <c r="Q4" s="2" t="n"/>
       <c r="R4" s="2" t="n"/>
       <c r="S4" s="2" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>LNZ:VIE</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Lenzing AG</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>equity</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Fast</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>254</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>3048.97</v>
+      </c>
+      <c r="I5" s="5" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="n">
+        <v>3036.82</v>
+      </c>
+      <c r="L5" s="3" t="n">
+        <v>-12.15</v>
+      </c>
+      <c r="M5" s="4" t="n">
+        <v>-0.004</v>
+      </c>
+      <c r="N5" s="4" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="O5" s="5" t="n">
+        <v>12.9</v>
+      </c>
+      <c r="P5" s="4" t="n">
+        <v>0.2056</v>
+      </c>
+      <c r="Q5" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-09</t>
+        </is>
+      </c>
+      <c r="R5" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="S5" s="2" t="inlineStr">
+        <is>
+          <t>Q3 EBITDA &lt; EUR90m; further capital/covenant event; user rules hybrids count as debt; mandatory exit 2026-12-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>PNN:LSE</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Pennon Group</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>equity</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>gated</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Fast</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="3" t="n"/>
+      <c r="I6" s="5" t="n"/>
+      <c r="J6" s="2" t="n"/>
+      <c r="K6" s="3" t="n"/>
+      <c r="L6" s="3" t="n"/>
+      <c r="M6" s="4" t="n"/>
+      <c r="N6" s="4" t="n"/>
+      <c r="O6" s="5" t="n"/>
+      <c r="P6" s="4" t="n"/>
+      <c r="Q6" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="R6" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="S6" s="2" t="inlineStr">
+        <is>
+          <t>n/a until user rules on regulated-utility leverage (memo W44 q1); Yahoo quotes in pence</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>ERA:PAR</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Eramet</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>equity</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>watchlist</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Fast</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="3" t="n"/>
+      <c r="I7" s="5" t="n"/>
+      <c r="J7" s="2" t="n"/>
+      <c r="K7" s="3" t="n"/>
+      <c r="L7" s="3" t="n"/>
+      <c r="M7" s="4" t="n"/>
+      <c r="N7" s="4" t="n"/>
+      <c r="O7" s="5" t="n"/>
+      <c r="P7" s="4" t="n"/>
+      <c r="Q7" s="2" t="n"/>
+      <c r="R7" s="2" t="n"/>
+      <c r="S7" s="2" t="inlineStr">
+        <is>
+          <t>n/a until prospectus; leverage test on prospectus balance sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>YCA:AIM</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Yellow Cake plc</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>equity</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>watchlist</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Fast</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="3" t="n"/>
+      <c r="I8" s="5" t="n"/>
+      <c r="J8" s="2" t="n"/>
+      <c r="K8" s="3" t="n"/>
+      <c r="L8" s="3" t="n"/>
+      <c r="M8" s="4" t="n"/>
+      <c r="N8" s="4" t="n"/>
+      <c r="O8" s="5" t="n"/>
+      <c r="P8" s="4" t="n"/>
+      <c r="Q8" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-30</t>
+        </is>
+      </c>
+      <c r="R8" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="S8" s="2" t="inlineStr">
+        <is>
+          <t>n/a until final list and NAV discount checked; Yahoo quotes in pence</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2504,7 +2793,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2688,6 +2977,60 @@
       <c r="L3" s="2" t="inlineStr">
         <is>
           <t>ATSE close 21 Oct 2026 per Yahoo (backfill); memo W43 used the Stuttgart quote 13.94 as proxy on decision day</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>2026-W44</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>LNZ:VIE</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>254</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" s="5" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>1.117381</v>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Stock 29% below TERP (EUR15.04) eight days after a 99%-subscribed 9-for-10 rights issue at EUR8.65; selling was discretionary and ATX flow is a buyer; fast sleeve 3% of NAV</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>2026-W44.md</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>Vienna close 28 Oct 2026 per boerse-social.com entered as manual row; Yahoo unreachable from routine sandbox; EURUSD 27 Oct feed close</t>
         </is>
       </c>
     </row>
@@ -2744,7 +3087,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3001,6 +3344,308 @@
       </c>
       <c r="N4" s="2" t="n"/>
     </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Lenzing</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>LNZ:VIE</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="n">
+        <v>12.9</v>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Post-rights overhang clearance (TERP 15.04); Q3 5 Nov</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-09</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Q3 EBITDA &lt; EUR90m; further capital/covenant event; hybrid ruling; mandatory exit 9 Dec</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>n/a (fast sleeve)</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>2026-W44.md</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Pennon</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>PNN:LSE</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>352</v>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>GBp</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="n"/>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Post-rights overhang (TERP 387.73p; rump 330p); H1 results 1 Dec 2026</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>n/a until ruling</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>W48</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>gated</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>2026-W44.md</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>Gated on leverage exclusion (7.4x ND/EBITDA pro forma); memo W44 q1</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Eramet</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>ERA:PAR</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>34</v>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="n"/>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>EUR500m rights issue with State backstop; terms after 29 Oct Q3 release</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="n"/>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>n/a until prospectus</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="n"/>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>watchlist</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>2026-W44.md</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>Price 26 Oct close (MarketScreener); adjusted leverage 4.5x at H1; entry only during/after rights period</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Yellow Cake</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>YCA:AIM</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>562</v>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>GBp</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="n"/>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>MSCI non-operating-company deletion; list 11 Nov; effective 30 Nov</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-30</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>n/a until list and NAV discount</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>W48</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>watchlist</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>2026-W44.md</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>Price stale (13 Aug 2026 UNVERIFIED); NAV not retrieved; memo W44 q3</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Corteva</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>CTVA:NYSE</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>11.63</v>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="n"/>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Parent after Vylor spin (1 Oct); S&amp;P 500 to MidCap 400 on 6 Oct; at 52-week low</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="n"/>
+      <c r="J9" s="2" t="n"/>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>W48</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>pointer</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>2026-W44.md</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>Lens-0 pointer for W48; US-situs; price 27 Oct close (stockanalysis.com)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3012,7 +3657,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3198,6 +3843,156 @@
       <c r="F6" s="2" t="inlineStr">
         <is>
           <t>A dated regulatory decision</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Genting Berhad</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>GENTING:KLSE</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>RM1.25bn rights issue partly funds interest and short-term debt repayment at a levered holdco; Bursa access at IBKR unverified</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Never while proceeds fund interest</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Raizen</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>RAIZ4:B3</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Distressed recap inside recuperacao extrajudicial; net debt R$60bn vs market cap about R$3bn; Brazil cap; lens-1 question only after conversion</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Post-conversion balance sheet below 2.5x and a dated event</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Unipol Assicurazioni</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>UNI:MIL</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Financial (insurer buying bank branches); stock rose on announcement; no overhang</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Never (financial exclusion)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Strategy / Metaplanet</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>MSTR:NASDAQ and 3350:TSE</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Likely MSCI deletions 30 Nov but leveraged bitcoin holding vehicles; excluded on substance</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Never</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Oncoclinicas (follow-up)</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>ONCO3:B3</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>OPA suspended by federal injunction 23 Oct 2026 one day before CVM deadline; merits undecided; no dated event</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Injunction lifted and an edital de OPA with a leilao date</t>
         </is>
       </c>
     </row>
@@ -3327,7 +4122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F281"/>
+  <dimension ref="A1:F282"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -11038,6 +11833,36 @@
         </is>
       </c>
     </row>
+    <row r="282">
+      <c r="A282" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B282" s="2" t="inlineStr">
+        <is>
+          <t>LNZ.VI</t>
+        </is>
+      </c>
+      <c r="C282" s="5" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="D282" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="E282" s="2" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="F282" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>